<commit_message>
docs(entrega): cobertura 100%, matriz y casos de prueba actualizados, LEEME alineado
</commit_message>
<xml_diff>
--- a/entregables/casos_y_trazabilidad/Matriz_de_Trazabilidad.xlsx
+++ b/entregables/casos_y_trazabilidad/Matriz_de_Trazabilidad.xlsx
@@ -669,7 +669,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:D97"/>
+  <dimension ref="A1:D104"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.6171875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12.28" customWidth="1" style="21" min="1" max="1"/>
@@ -741,7 +741,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>381, 382, 670, 671</t>
+          <t>463, 464, 816, 817</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>383, 384, 674, 675, 676, 677</t>
+          <t>465, 466, 467, 820, 821, 822, 823, 824</t>
         </is>
       </c>
     </row>
@@ -781,7 +781,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>385, 386, 387, 388, 696, 697, 698, 699</t>
+          <t>468, 469, 470, 471, 472, 843, 844, 845, 846</t>
         </is>
       </c>
     </row>
@@ -801,7 +801,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>389, 390, 391, 392, 393, 394, 395, 396, 397, 398, 399, 400, 401, 402, 403</t>
+          <t>473, 474, 475, 476, 477, 478, 479, 480, 481, 482, 483, 484, 485, 486, 487, 488</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>404, 405, 406, 707, 708, 709</t>
+          <t>489, 490, 491, 492, 493, 854, 855, 856</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>407, 408, 409, 410, 411, 710, 711</t>
+          <t>494, 495, 496, 497, 498, 499, 500, 857, 858</t>
         </is>
       </c>
     </row>
@@ -861,7 +861,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>412, 714</t>
+          <t>501, 861</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>667, 668, 669</t>
+          <t>813, 814, 815</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>672</t>
+          <t>818</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>673</t>
+          <t>819</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>678, 679, 680, 681</t>
+          <t>825, 826, 827, 828</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>682, 683</t>
+          <t>829, 830</t>
         </is>
       </c>
     </row>
@@ -981,7 +981,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>684, 685, 686, 687, 688, 689</t>
+          <t>831, 832, 833, 834, 835, 836</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>690, 691, 692, 693, 694, 695</t>
+          <t>837, 838, 839, 840, 841, 842</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>700, 701, 702, 703, 704, 705, 706</t>
+          <t>847, 848, 849, 850, 851, 852, 853</t>
         </is>
       </c>
     </row>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>712, 713</t>
+          <t>859, 860</t>
         </is>
       </c>
     </row>
@@ -1061,7 +1061,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>350, 351, 352, 353, 354, 355, 356, 357, 358, 359, 360</t>
+          <t>432, 433, 434, 435, 436, 437, 438, 439, 440, 441, 442</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>361, 362, 363, 364, 365, 366, 367, 368, 369, 370, 371, 372, 373, 374, 375, 376, 377, 378, 379, 380</t>
+          <t>443, 444, 445, 446, 447, 448, 449, 450, 451, 452, 453, 454, 455, 456, 457, 458, 459, 460, 461, 462</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>654, 655, 656, 657, 658, 659, 660, 661</t>
+          <t>798, 799, 800, 801, 802, 803, 804, 805, 806, 807</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>662, 663, 664, 665, 666</t>
+          <t>808, 809, 810, 811, 812</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>313, 314, 315, 316, 317, 318, 319, 320, 321, 322, 323, 324, 325, 326</t>
+          <t>384, 385, 386, 387, 388, 389, 390, 391, 392, 393, 394, 395, 396, 397, 398, 399</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>327, 328, 329, 330, 331, 332, 333, 334, 335, 336, 337, 338, 339, 340, 341, 342, 343, 344, 345, 346, 347, 348, 349</t>
+          <t>400, 401, 402, 403, 404, 405, 406, 407, 408, 409, 410, 411, 412, 413, 414, 415, 416, 417, 418, 419, 420, 421, 422, 423, 424, 425, 426, 427, 428, 429, 430, 431</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>612, 613, 614, 615, 616, 617, 618, 619, 620, 621, 622, 623, 624, 625, 626, 627, 628, 629, 630, 631, 632, 633</t>
+          <t>743, 744, 745, 746, 747, 748, 749, 750, 751, 752, 753, 754, 755, 756, 757, 758, 759, 760, 761, 762, 763, 764, 765, 766, 767, 768, 769</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>634, 635, 636, 637, 638, 639, 640, 641, 642, 643</t>
+          <t>770, 771, 772, 773, 774, 775, 776, 777, 778, 779, 780, 781, 782, 783, 784, 785, 786, 787</t>
         </is>
       </c>
     </row>
@@ -1221,7 +1221,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>644, 645, 646, 647, 648, 649, 650, 651, 652, 653</t>
+          <t>788, 789, 790, 791, 792, 793, 794, 795, 796, 797</t>
         </is>
       </c>
     </row>
@@ -1241,7 +1241,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>527, 528, 529, 530, 531, 532, 533, 534, 535, 536, 537, 538, 539, 540, 541, 542</t>
+          <t>636, 637, 638, 639, 640, 641, 642, 643, 644, 645, 646, 647, 648, 649, 650, 651, 652, 653</t>
         </is>
       </c>
     </row>
@@ -1251,17 +1251,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>US_5: Plantillas y generación de PDF (RF-03, CU-09)</t>
+          <t>US_4: Formularios dinámicos por tipo (RF-02)</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>T27: Bdd pdf</t>
+          <t>T27: Validators</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>202, 203</t>
+          <t>654, 655, 656, 657, 658, 659</t>
         </is>
       </c>
     </row>
@@ -1276,12 +1276,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>T28: Pdf service</t>
+          <t>T28: Bdd pdf</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>204, 205, 206, 207, 208, 209, 210, 211, 212, 213, 214, 215, 216</t>
+          <t>212, 213</t>
         </is>
       </c>
     </row>
@@ -1296,12 +1296,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>T29: Plantilla repository</t>
+          <t>T29: Pdf service</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>217, 218, 219, 220, 221, 222, 223, 224</t>
+          <t>214, 215, 216, 217, 218, 219, 220, 221, 222, 223, 224, 225, 226, 227, 228, 229, 230</t>
         </is>
       </c>
     </row>
@@ -1316,12 +1316,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>T30: Views</t>
+          <t>T30: Plantilla repository</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>225, 226, 227, 228, 229, 230, 231, 232, 233, 234, 235, 236, 237, 238, 239, 240, 241, 242</t>
+          <t>231, 232, 233, 234, 235, 236, 237, 238</t>
         </is>
       </c>
     </row>
@@ -1336,12 +1336,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>T31: Context</t>
+          <t>T31: Views</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>560, 561, 562, 563, 564, 565</t>
+          <t>239, 240, 241, 242, 243, 244, 245, 246, 247, 248, 249, 250, 251, 252, 253, 254, 255, 256, 257, 258, 259, 260, 261, 262, 263, 264, 265, 266, 267, 268, 269, 270, 271, 272, 273, 274, 275, 276, 277, 278</t>
         </is>
       </c>
     </row>
@@ -1356,12 +1356,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>T32: Exceptions</t>
+          <t>T32: Context</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>566, 567, 568</t>
+          <t>680, 681, 682, 683, 684, 685, 686, 687</t>
         </is>
       </c>
     </row>
@@ -1376,12 +1376,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>T33: Plantilla service</t>
+          <t>T33: Exceptions</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>569, 570, 571, 572</t>
+          <t>688, 689, 690</t>
         </is>
       </c>
     </row>
@@ -1396,12 +1396,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>T34: Schemas</t>
+          <t>T34: Plantilla service</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>573, 574, 575, 576, 577, 578, 579, 580, 581</t>
+          <t>691, 692, 693, 694</t>
         </is>
       </c>
     </row>
@@ -1411,17 +1411,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>US_6: Biblioteca de imágenes para plantillas</t>
+          <t>US_5: Plantillas y generación de PDF (RF-03, CU-09)</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>T35: Repositories</t>
+          <t>T35: Schemas</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>243, 244, 245, 246, 247, 248, 249, 250, 251, 252, 253</t>
+          <t>695, 696, 697, 698, 699, 700, 701, 702, 703</t>
         </is>
       </c>
     </row>
@@ -1436,12 +1436,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>T36: Views</t>
+          <t>T36: Repositories</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>254, 255, 256, 257, 258, 259, 260, 261, 262</t>
+          <t>279, 280, 281, 282, 283, 284, 285, 286, 287, 288, 289, 290, 291, 292</t>
         </is>
       </c>
     </row>
@@ -1456,12 +1456,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>T37: Forms</t>
+          <t>T37: Views</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>582, 583, 584, 585</t>
+          <t>293, 294, 295, 296, 297, 298, 299, 300, 301, 302, 303, 304, 305, 306, 307, 308, 309, 310, 311, 312, 313, 314, 315, 316, 522</t>
         </is>
       </c>
     </row>
@@ -1476,12 +1476,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>T38: Services</t>
+          <t>T38: Forms</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>586, 587, 588, 589, 590, 591, 592</t>
+          <t>704, 705, 706, 707, 708, 709</t>
         </is>
       </c>
     </row>
@@ -1491,17 +1491,17 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>US_7: Creación de solicitudes por el solicitante (RF-04)</t>
+          <t>US_6: Biblioteca de imágenes para plantillas</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>T39: Bdd intake</t>
+          <t>T39: Services</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>127, 128</t>
+          <t>710, 711, 712, 713, 714, 715, 716, 717, 718</t>
         </is>
       </c>
     </row>
@@ -1516,12 +1516,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>T40: E2e tier1</t>
+          <t>T40: Bdd intake</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>129, 130, 131, 132</t>
+          <t>134, 135</t>
         </is>
       </c>
     </row>
@@ -1536,12 +1536,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>T41: Intake service</t>
+          <t>T41: E2e tier1</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>133, 134, 135, 136, 137, 138, 139, 140</t>
+          <t>136, 137, 138, 139</t>
         </is>
       </c>
     </row>
@@ -1556,12 +1556,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>T42: Intake views</t>
+          <t>T42: Intake service</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>141, 142, 143, 144, 145, 146, 147, 148, 149, 150, 151, 152, 153, 154, 155, 156, 157</t>
+          <t>140, 141, 142, 143, 144, 145, 146, 147</t>
         </is>
       </c>
     </row>
@@ -1576,12 +1576,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>T43: Auto fill resolver</t>
+          <t>T43: Intake views</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>543, 544, 545, 546, 547, 548, 549, 550, 551</t>
+          <t>148, 149, 150, 151, 152, 153, 154, 155, 156, 157, 158, 159, 160, 161, 162, 163, 164, 165, 166</t>
         </is>
       </c>
     </row>
@@ -1591,17 +1591,17 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
+          <t>US_7: Creación de solicitudes por el solicitante (RF-04)</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>T44: Folio repository</t>
+          <t>T44: Auto fill resolver</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>158, 159, 160</t>
+          <t>660, 661, 662, 663, 664, 665, 666, 667, 668</t>
         </is>
       </c>
     </row>
@@ -1611,17 +1611,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
+          <t>US_7: Creación de solicitudes por el solicitante (RF-04)</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>T45: Historial repository</t>
+          <t>T45: Mentor port</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>161, 162, 163, 164</t>
+          <t>669</t>
         </is>
       </c>
     </row>
@@ -1636,12 +1636,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>T46: Lifecycle service</t>
+          <t>T46: Folio repository</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>165, 166, 167, 168, 169, 170, 171, 172, 173, 174, 175, 176, 177</t>
+          <t>167, 168, 169</t>
         </is>
       </c>
     </row>
@@ -1656,12 +1656,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>T47: Solicitud repository</t>
+          <t>T47: Historial repository</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>178, 179, 180, 181, 182, 183, 184, 185, 186, 187, 188, 189, 190, 191, 192, 193, 194, 195, 196</t>
+          <t>170, 171, 172, 173</t>
         </is>
       </c>
     </row>
@@ -1676,12 +1676,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>T48: Solicitud repository aggregates</t>
+          <t>T48: Lifecycle service</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>197, 198, 199, 200, 201</t>
+          <t>174, 175, 176, 177, 178, 179, 180, 181, 182, 183, 184, 185, 186</t>
         </is>
       </c>
     </row>
@@ -1696,12 +1696,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>T49: Folio service</t>
+          <t>T49: Solicitud repository</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>552, 553</t>
+          <t>187, 188, 189, 190, 191, 192, 193, 194, 195, 196, 197, 198, 199, 200, 201, 202, 203, 204, 205, 206</t>
         </is>
       </c>
     </row>
@@ -1716,12 +1716,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>T50: Lifecycle service aggregates</t>
+          <t>T50: Solicitud repository aggregates</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>554, 555, 556, 557, 558, 559</t>
+          <t>207, 208, 209, 210, 211</t>
         </is>
       </c>
     </row>
@@ -1731,17 +1731,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>US_9: Cola de revisión y atención por rol (RF-06, RF-09)</t>
+          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>T51: Bdd revision</t>
+          <t>T51: Folio service</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>298, 299</t>
+          <t>670, 671</t>
         </is>
       </c>
     </row>
@@ -1751,17 +1751,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>US_9: Cola de revisión y atención por rol (RF-06, RF-09)</t>
+          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>T52: Revision views</t>
+          <t>T52: Lifecycle service aggregates</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>300, 301, 302, 303, 304, 305, 306, 307, 308, 309, 310, 311, 312</t>
+          <t>672, 673, 674, 675, 676, 677</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1771,17 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
+          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>T53: Repository</t>
+          <t>T53: Notification port</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>263, 264, 265, 266, 267, 268, 604</t>
+          <t>678, 679</t>
         </is>
       </c>
     </row>
@@ -1791,17 +1791,17 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
+          <t>US_9: Cola de revisión y atención por rol (RF-06, RF-09)</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>T54: Service</t>
+          <t>T54: Bdd revision</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>269, 270, 271, 272, 273, 274, 275, 276, 277, 278, 279, 280, 281, 282, 283, 284, 285, 286, 287, 288</t>
+          <t>353, 354</t>
         </is>
       </c>
     </row>
@@ -1811,17 +1811,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
+          <t>US_9: Cola de revisión y atención por rol (RF-06, RF-09)</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>T55: Views</t>
+          <t>T55: Revision views</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>289, 290, 291, 292, 293, 294, 295, 296, 297</t>
+          <t>355, 356, 357, 358, 359, 360, 361, 362, 363, 364, 365, 366, 367, 368, 369, 370, 371, 372, 373</t>
         </is>
       </c>
     </row>
@@ -1836,12 +1836,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>T56: Exceptions</t>
+          <t>T56: Repository</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>593, 594, 595, 596, 597, 598</t>
+          <t>317, 318, 319, 320, 321, 322, 731</t>
         </is>
       </c>
     </row>
@@ -1856,12 +1856,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>T57: Forms</t>
+          <t>T57: Service</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>599, 600, 601, 602, 603</t>
+          <t>323, 324, 325, 326, 327, 328, 329, 330, 331, 332, 333, 334, 335, 336, 337, 338, 339, 340, 341, 342, 343</t>
         </is>
       </c>
     </row>
@@ -1876,12 +1876,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>T58: Schemas</t>
+          <t>T58: Views</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>605, 606, 607, 608, 609, 610, 611</t>
+          <t>344, 345, 346, 347, 348, 349, 350, 351, 352</t>
         </is>
       </c>
     </row>
@@ -1891,17 +1891,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
+          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>T59: Archivo service</t>
+          <t>T59: Exceptions</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>107, 108, 511, 512, 513, 514, 515, 516, 517, 518, 519, 520, 521, 522, 523, 524, 525</t>
+          <t>719, 720, 721, 722, 723, 724</t>
         </is>
       </c>
     </row>
@@ -1911,17 +1911,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
+          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>T60: Bdd archivos</t>
+          <t>T60: Forms</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>109, 110</t>
+          <t>725, 726, 727, 728, 729, 730</t>
         </is>
       </c>
     </row>
@@ -1931,17 +1931,17 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
+          <t>US_10: Respuesta de la institución y archivos de respuesta (RF-09)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>T61: Download view</t>
+          <t>T61: Schemas</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>111, 112, 113, 114, 115</t>
+          <t>732, 733, 734, 735, 736, 737, 738</t>
         </is>
       </c>
     </row>
@@ -1956,12 +1956,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>T62: Repository</t>
+          <t>T62: Archivo service</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>116, 117, 118, 119, 120, 121, 122, 123, 124, 125, 126</t>
+          <t>114, 115, 507, 508, 509, 615, 616, 617, 618, 619, 620, 621, 622, 623, 624, 625, 626, 627, 628, 629, 630, 631, 632, 633</t>
         </is>
       </c>
     </row>
@@ -1976,12 +1976,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>T63: E2e tier1</t>
+          <t>T63: Bdd archivos</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>418, 419, 420, 421, 422</t>
+          <t>116, 117</t>
         </is>
       </c>
     </row>
@@ -1996,12 +1996,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>T64: Local storage</t>
+          <t>T64: Download view</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>423, 424, 425, 426, 427, 526</t>
+          <t>118, 119, 120, 121, 122</t>
         </is>
       </c>
     </row>
@@ -2011,17 +2011,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
+          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>T65: Bdd catalogo</t>
+          <t>T65: Repository</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>10, 11, 12</t>
+          <t>123, 124, 125, 126, 127, 128, 129, 130, 131, 132, 133</t>
         </is>
       </c>
     </row>
@@ -2031,17 +2031,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
+          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>T66: Csv importer</t>
+          <t>T66: E2e tier1</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>13, 14, 15, 16, 17, 18, 19, 20, 21, 22, 23</t>
+          <t>510, 511, 512, 513, 514</t>
         </is>
       </c>
     </row>
@@ -2051,17 +2051,17 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
+          <t>US_11: Gestión de archivos adjuntos (RF-10)</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>T67: Intake wiring</t>
+          <t>T67: Local storage</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>24, 25, 26, 27, 28, 29, 30</t>
+          <t>515, 516, 517, 518, 519, 520, 521, 634, 635</t>
         </is>
       </c>
     </row>
@@ -2076,12 +2076,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>T68: Mentor repository</t>
+          <t>T68: Bdd catalogo</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>31, 32, 33, 34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 415, 416, 417</t>
+          <t>12, 13, 14</t>
         </is>
       </c>
     </row>
@@ -2096,12 +2096,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>T69: Views</t>
+          <t>T69: Csv importer</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>55, 56, 57, 58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84</t>
+          <t>15, 16, 17, 18, 19, 20, 21, 22, 23, 24, 25</t>
         </is>
       </c>
     </row>
@@ -2116,12 +2116,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>T70: Backfill migration</t>
+          <t>T70: Forms models</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>413, 414</t>
+          <t>26, 566, 567</t>
         </is>
       </c>
     </row>
@@ -2136,12 +2136,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>T71: Mentor service</t>
+          <t>T71: Intake wiring</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>464, 465, 466, 467, 468, 469, 470, 471, 472, 473, 474, 475, 476, 477, 478, 479, 480</t>
+          <t>27, 28, 29, 30, 31, 32, 33</t>
         </is>
       </c>
     </row>
@@ -2151,17 +2151,17 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
+          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>T72: Bdd dispatch</t>
+          <t>T72: Mentor repository</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>85, 86</t>
+          <t>34, 35, 36, 37, 38, 39, 40, 41, 42, 43, 44, 45, 46, 47, 48, 49, 50, 51, 52, 53, 54, 55, 56, 57, 504, 505, 506</t>
         </is>
       </c>
     </row>
@@ -2171,17 +2171,17 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
+          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>T73: E2e tier1</t>
+          <t>T73: Views</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>87, 88, 89, 90</t>
+          <t>58, 59, 60, 61, 62, 63, 64, 65, 66, 67, 68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80, 81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91</t>
         </is>
       </c>
     </row>
@@ -2191,17 +2191,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
+          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>T74: Email sender</t>
+          <t>T74: Backfill migration</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>91, 481, 482</t>
+          <t>502, 503</t>
         </is>
       </c>
     </row>
@@ -2211,17 +2211,17 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
+          <t>US_12: Gestión de alumnos mentores e importación CSV (RF-11)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>T75: Notification service</t>
+          <t>T75: Mentor service</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>483, 484, 485, 486, 487, 488</t>
+          <t>568, 569, 570, 571, 572, 573, 574, 575, 576, 577, 578, 579, 580, 581, 582, 583, 584</t>
         </is>
       </c>
     </row>
@@ -2236,12 +2236,12 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>T76: Recipient resolver</t>
+          <t>T76: Bdd dispatch</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>489, 490</t>
+          <t>92, 93</t>
         </is>
       </c>
     </row>
@@ -2251,17 +2251,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
+          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>T77: Bdd dashboard</t>
+          <t>T77: E2e tier1</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>92, 93, 94</t>
+          <t>94, 95, 96, 97</t>
         </is>
       </c>
     </row>
@@ -2271,17 +2271,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
+          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>T78: Views</t>
+          <t>T78: Email sender</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>95, 96, 97, 98, 99, 100, 101, 102, 103, 104, 105, 106</t>
+          <t>98, 585, 586</t>
         </is>
       </c>
     </row>
@@ -2291,17 +2291,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
+          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>T79: Csv exporter</t>
+          <t>T79: Notification service</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>491, 492, 493</t>
+          <t>587, 588, 589, 590, 591, 592</t>
         </is>
       </c>
     </row>
@@ -2311,17 +2311,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
+          <t>US_13: Notificaciones por correo en el ciclo de vida (RF-07)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>T80: Pdf exporter</t>
+          <t>T80: Recipient resolver</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>494, 495, 496, 497</t>
+          <t>593, 594</t>
         </is>
       </c>
     </row>
@@ -2336,12 +2336,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>T81: Report filter form</t>
+          <t>T81: Bdd dashboard</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>498, 499, 500, 501, 502, 503, 504, 505</t>
+          <t>99, 100, 101</t>
         </is>
       </c>
     </row>
@@ -2356,12 +2356,12 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>T82: Report service</t>
+          <t>T82: Views</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>506, 507, 508, 509, 510</t>
+          <t>102, 103, 104, 105, 106, 107, 108, 109, 110, 111, 112, 113</t>
         </is>
       </c>
     </row>
@@ -2371,17 +2371,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>T83: Home view</t>
+          <t>T83: Csv exporter</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>1, 2, 437</t>
+          <t>595, 596, 597</t>
         </is>
       </c>
     </row>
@@ -2391,17 +2391,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>T84: Seed command</t>
+          <t>T84: Pdf exporter</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>3, 4, 5, 6, 7, 8, 9</t>
+          <t>598, 599, 600, 601</t>
         </is>
       </c>
     </row>
@@ -2411,17 +2411,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>T85: Audit</t>
+          <t>T85: Report filter form</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>428</t>
+          <t>602, 603, 604, 605, 606, 607, 608, 609</t>
         </is>
       </c>
     </row>
@@ -2431,17 +2431,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+          <t>US_14: Dashboard administrativo y exportación de reportes (CU-14, CU-15)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>T86: Auth</t>
+          <t>T86: Report service</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>429, 430, 431, 432</t>
+          <t>610, 611, 612, 613, 614</t>
         </is>
       </c>
     </row>
@@ -2456,12 +2456,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>T87: Exceptions</t>
+          <t>T87: Home view</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>433, 434, 435, 436</t>
+          <t>1, 2, 532, 533</t>
         </is>
       </c>
     </row>
@@ -2476,12 +2476,12 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>T88: Lucide tag</t>
+          <t>T88: Seed command</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>438, 439, 440, 441</t>
+          <t>3, 4, 5, 6, 7, 8, 9, 10, 11</t>
         </is>
       </c>
     </row>
@@ -2496,12 +2496,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>T89: Middleware error handler</t>
+          <t>T89: Audit</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>442, 443, 444, 445, 446, 447, 448</t>
+          <t>523</t>
         </is>
       </c>
     </row>
@@ -2516,12 +2516,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>T90: Middleware logging</t>
+          <t>T90: Auth</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>449</t>
+          <t>524, 525, 526, 527</t>
         </is>
       </c>
     </row>
@@ -2536,12 +2536,12 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>T91: Middleware request id</t>
+          <t>T91: Exceptions</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>450, 451, 452, 453, 454</t>
+          <t>528, 529, 530, 531</t>
         </is>
       </c>
     </row>
@@ -2556,12 +2556,12 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>T92: Pagination</t>
+          <t>T92: Lucide tag</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>455, 456, 457, 458, 459, 460, 461</t>
+          <t>534, 535, 536, 537, 538</t>
         </is>
       </c>
     </row>
@@ -2576,12 +2576,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>T93: Pdf</t>
+          <t>T93: Middleware error handler</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>462</t>
+          <t>539, 540, 541, 542, 543, 544, 545</t>
         </is>
       </c>
     </row>
@@ -2596,22 +2596,155 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>T94: Static assets</t>
+          <t>T94: Middleware logging</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>463</t>
-        </is>
-      </c>
-    </row>
-    <row r="98" ht="15.75" customHeight="1" s="22"/>
-    <row r="99" ht="15.75" customHeight="1" s="22"/>
-    <row r="100" ht="15.75" customHeight="1" s="22"/>
-    <row r="101" ht="15.75" customHeight="1" s="22"/>
-    <row r="102" ht="15.75" customHeight="1" s="22"/>
-    <row r="103" ht="15.75" customHeight="1" s="22"/>
-    <row r="104" ht="15.75" customHeight="1" s="22"/>
+          <t>546, 547, 548</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="15.75" customHeight="1" s="22">
+      <c r="A98" t="n">
+        <v>95</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>T95: Middleware request id</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>549, 550, 551, 552, 553</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="15.75" customHeight="1" s="22">
+      <c r="A99" t="n">
+        <v>96</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>T96: Pagination</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>554, 555, 556, 557, 558, 559, 560, 561</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="15.75" customHeight="1" s="22">
+      <c r="A100" t="n">
+        <v>97</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>T97: Pdf</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>562</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="15.75" customHeight="1" s="22">
+      <c r="A101" t="n">
+        <v>98</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>T98: Request actor</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>563, 564</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="15.75" customHeight="1" s="22">
+      <c r="A102" t="n">
+        <v>99</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>US_15: Infraestructura compartida (auth, manejo de errores, auditoría, PDF)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>T99: Static assets</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>565</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="15.75" customHeight="1" s="22">
+      <c r="A103" t="n">
+        <v>100</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>T100: Models str</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>374, 375, 376, 377, 378, 379, 380, 381, 382, 383</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="15.75" customHeight="1" s="22">
+      <c r="A104" t="n">
+        <v>101</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>US_8: Ciclo de vida y transiciones de la solicitud (RF-05)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>T101: Templatetags</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>739, 740, 741, 742</t>
+        </is>
+      </c>
+    </row>
     <row r="105" ht="15.75" customHeight="1" s="22"/>
     <row r="106" ht="15.75" customHeight="1" s="22"/>
     <row r="107" ht="15.75" customHeight="1" s="22"/>

</xml_diff>